<commit_message>
Look at it in Excel
</commit_message>
<xml_diff>
--- a/lexicon/lexicon.xlsx
+++ b/lexicon/lexicon.xlsx
@@ -1673,8 +1673,10 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
-        <v>5</v>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">afraid</t>
+        </is>
       </c>
       <c r="B2" s="2" t="s">
         <v>324</v>
@@ -1687,8 +1689,10 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>7</v>
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">all</t>
+        </is>
       </c>
       <c r="B3" s="2" t="s">
         <v>8</v>
@@ -1701,8 +1705,10 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>10</v>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">basket</t>
+        </is>
       </c>
       <c r="B4" s="2" t="s">
         <v>11</v>
@@ -1715,8 +1721,10 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
-        <v>13</v>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">big</t>
+        </is>
       </c>
       <c r="B5" s="2" t="s">
         <v>14</v>
@@ -1732,8 +1740,10 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
-        <v>16</v>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bird</t>
+        </is>
       </c>
       <c r="B6" s="2" t="s">
         <v>322</v>
@@ -1746,8 +1756,10 @@
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
-        <v>18</v>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">black</t>
+        </is>
       </c>
       <c r="B7" s="2" t="s">
         <v>19</v>
@@ -1763,8 +1775,10 @@
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
-        <v>21</v>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">blackberry</t>
+        </is>
       </c>
       <c r="B8" s="2" t="s">
         <v>22</v>
@@ -1777,8 +1791,10 @@
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A9" s="3" t="s">
-        <v>24</v>
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bone-game</t>
+        </is>
       </c>
       <c r="B9" s="2" t="s">
         <v>25</v>
@@ -1791,8 +1807,10 @@
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A10" s="3" t="s">
-        <v>28</v>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bread</t>
+        </is>
       </c>
       <c r="B10" s="2" t="s">
         <v>29</v>
@@ -1805,8 +1823,10 @@
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A11" s="3" t="s">
-        <v>31</v>
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">canoe</t>
+        </is>
       </c>
       <c r="B11" s="2" t="s">
         <v>32</v>
@@ -1822,8 +1842,10 @@
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A12" s="3" t="s">
-        <v>34</v>
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cat</t>
+        </is>
       </c>
       <c r="B12" s="2" t="s">
         <v>35</v>
@@ -1839,8 +1861,10 @@
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A13" s="3" t="s">
-        <v>37</v>
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cedar-wood</t>
+        </is>
       </c>
       <c r="B13" s="2" t="s">
         <v>38</v>
@@ -1853,8 +1877,10 @@
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A14" s="3" t="s">
-        <v>41</v>
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">chinook-salmon</t>
+        </is>
       </c>
       <c r="B14" s="2" t="s">
         <v>42</v>
@@ -1867,8 +1893,10 @@
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A15" s="3" t="s">
-        <v>45</v>
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">coat</t>
+        </is>
       </c>
       <c r="B15" s="2" t="s">
         <v>46</v>
@@ -1881,8 +1909,10 @@
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A16" s="3" t="s">
-        <v>48</v>
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">comb</t>
+        </is>
       </c>
       <c r="B16" s="2" t="s">
         <v>49</v>
@@ -1895,8 +1925,10 @@
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A17" s="3" t="s">
-        <v>51</v>
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">continue</t>
+        </is>
       </c>
       <c r="B17" s="2" t="s">
         <v>52</v>
@@ -1909,8 +1941,10 @@
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A18" s="3" t="s">
-        <v>54</v>
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cow</t>
+        </is>
       </c>
       <c r="B18" s="2" t="s">
         <v>55</v>
@@ -1923,8 +1957,10 @@
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A19" s="3" t="s">
-        <v>57</v>
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">crab</t>
+        </is>
       </c>
       <c r="B19" s="2" t="s">
         <v>58</v>
@@ -1937,8 +1973,10 @@
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A20" s="3" t="s">
-        <v>60</v>
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cry</t>
+        </is>
       </c>
       <c r="B20" s="2" t="s">
         <v>61</v>
@@ -1954,8 +1992,10 @@
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A21" s="3" t="s">
-        <v>63</v>
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cut-it</t>
+        </is>
       </c>
       <c r="B21" s="2" t="s">
         <v>323</v>
@@ -1971,8 +2011,10 @@
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A22" s="3" t="s">
-        <v>66</v>
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">day</t>
+        </is>
       </c>
       <c r="B22" s="2" t="s">
         <v>67</v>
@@ -1985,8 +2027,10 @@
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A23" s="3" t="s">
-        <v>69</v>
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">deer</t>
+        </is>
       </c>
       <c r="B23" s="2" t="s">
         <v>70</v>
@@ -2002,8 +2046,10 @@
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A24" s="3" t="s">
-        <v>72</v>
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dirt</t>
+        </is>
       </c>
       <c r="B24" s="2" t="s">
         <v>73</v>
@@ -2016,8 +2062,10 @@
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A25" s="3" t="s">
-        <v>75</v>
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">disappear</t>
+        </is>
       </c>
       <c r="B25" s="2" t="s">
         <v>76</v>
@@ -2030,8 +2078,10 @@
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A26" s="3" t="s">
-        <v>78</v>
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dog</t>
+        </is>
       </c>
       <c r="B26" s="2" t="s">
         <v>79</v>
@@ -2047,8 +2097,10 @@
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A27" s="3" t="s">
-        <v>81</v>
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">duck</t>
+        </is>
       </c>
       <c r="B27" s="2" t="s">
         <v>82</v>
@@ -2061,8 +2113,10 @@
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A28" s="3" t="s">
-        <v>84</v>
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ear</t>
+        </is>
       </c>
       <c r="B28" s="2" t="s">
         <v>85</v>
@@ -2075,8 +2129,10 @@
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A29" s="3" t="s">
-        <v>87</v>
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eat</t>
+        </is>
       </c>
       <c r="B29" s="2" t="s">
         <v>88</v>
@@ -2089,8 +2145,10 @@
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A30" s="3" t="s">
-        <v>90</v>
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">elwha</t>
+        </is>
       </c>
       <c r="B30" s="2" t="s">
         <v>91</v>
@@ -2103,8 +2161,10 @@
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A31" s="3" t="s">
-        <v>94</v>
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">enter</t>
+        </is>
       </c>
       <c r="B31" s="2" t="s">
         <v>95</v>
@@ -2117,8 +2177,10 @@
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A32" s="3" t="s">
-        <v>97</v>
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">evening</t>
+        </is>
       </c>
       <c r="B32" s="2" t="s">
         <v>98</v>
@@ -2131,8 +2193,10 @@
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A33" s="3" t="s">
-        <v>100</v>
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">finish</t>
+        </is>
       </c>
       <c r="B33" s="2" t="s">
         <v>101</v>
@@ -2145,8 +2209,10 @@
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A34" s="3" t="s">
-        <v>103</v>
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">five</t>
+        </is>
       </c>
       <c r="B34" s="2" t="s">
         <v>104</v>
@@ -2159,8 +2225,10 @@
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A35" s="3" t="s">
-        <v>106</v>
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">flip</t>
+        </is>
       </c>
       <c r="B35" s="2" t="s">
         <v>107</v>
@@ -2173,8 +2241,10 @@
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A36" s="3" t="s">
-        <v>109</v>
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">flounder</t>
+        </is>
       </c>
       <c r="B36" s="2" t="s">
         <v>110</v>
@@ -2187,8 +2257,10 @@
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A37" s="3" t="s">
-        <v>112</v>
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">foot</t>
+        </is>
       </c>
       <c r="B37" s="2" t="s">
         <v>113</v>
@@ -2201,8 +2273,10 @@
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A38" s="3" t="s">
-        <v>115</v>
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">four</t>
+        </is>
       </c>
       <c r="B38" s="2" t="s">
         <v>116</v>
@@ -2215,8 +2289,10 @@
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A39" s="3" t="s">
-        <v>118</v>
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">go</t>
+        </is>
       </c>
       <c r="B39" s="2" t="s">
         <v>119</v>
@@ -2232,8 +2308,10 @@
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A40" s="3" t="s">
-        <v>121</v>
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">go-home</t>
+        </is>
       </c>
       <c r="B40" s="2" t="s">
         <v>122</v>
@@ -2246,8 +2324,10 @@
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A41" s="3" t="s">
-        <v>125</v>
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">go-with</t>
+        </is>
       </c>
       <c r="B41" s="2" t="s">
         <v>126</v>
@@ -2260,8 +2340,10 @@
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A42" s="3" t="s">
-        <v>129</v>
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">good</t>
+        </is>
       </c>
       <c r="B42" s="2" t="s">
         <v>130</v>
@@ -2277,8 +2359,10 @@
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A43" s="3" t="s">
-        <v>132</v>
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">goodbye</t>
+        </is>
       </c>
       <c r="B43" s="2" t="s">
         <v>133</v>
@@ -2291,8 +2375,10 @@
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A44" s="3" t="s">
-        <v>135</v>
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hand</t>
+        </is>
       </c>
       <c r="B44" s="2" t="s">
         <v>136</v>
@@ -2305,8 +2391,10 @@
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A45" s="3" t="s">
-        <v>138</v>
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hat</t>
+        </is>
       </c>
       <c r="B45" s="2" t="s">
         <v>139</v>
@@ -2319,8 +2407,10 @@
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A46" s="3" t="s">
-        <v>141</v>
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">heart</t>
+        </is>
       </c>
       <c r="B46" s="2" t="s">
         <v>142</v>
@@ -2333,8 +2423,10 @@
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A47" s="3" t="s">
-        <v>144</v>
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">house</t>
+        </is>
       </c>
       <c r="B47" s="2" t="s">
         <v>145</v>
@@ -2350,8 +2442,10 @@
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A48" s="3" t="s">
-        <v>147</v>
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">how-many</t>
+        </is>
       </c>
       <c r="B48" s="2" t="s">
         <v>148</v>
@@ -2364,8 +2458,10 @@
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A49" s="3" t="s">
-        <v>151</v>
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hungry</t>
+        </is>
       </c>
       <c r="B49" s="2" t="s">
         <v>152</v>
@@ -2378,8 +2474,10 @@
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A50" s="3" t="s">
-        <v>154</v>
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">important-person</t>
+        </is>
       </c>
       <c r="B50" s="2" t="s">
         <v>155</v>
@@ -2392,8 +2490,10 @@
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A51" s="3" t="s">
-        <v>158</v>
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">jellyfish</t>
+        </is>
       </c>
       <c r="B51" s="2" t="s">
         <v>159</v>
@@ -2406,8 +2506,10 @@
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A52" s="3" t="s">
-        <v>161</v>
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">key</t>
+        </is>
       </c>
       <c r="B52" s="2" t="s">
         <v>162</v>
@@ -2420,8 +2522,10 @@
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A53" s="3" t="s">
-        <v>164</v>
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">know-it</t>
+        </is>
       </c>
       <c r="B53" s="2" t="s">
         <v>165</v>
@@ -2437,8 +2541,10 @@
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A54" s="3" t="s">
-        <v>168</v>
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">laugh</t>
+        </is>
       </c>
       <c r="B54" s="2" t="s">
         <v>169</v>
@@ -2451,8 +2557,10 @@
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A55" s="3" t="s">
-        <v>171</v>
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">like</t>
+        </is>
       </c>
       <c r="B55" s="2" t="s">
         <v>172</v>
@@ -2465,8 +2573,10 @@
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A56" s="3" t="s">
-        <v>174</v>
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">long</t>
+        </is>
       </c>
       <c r="B56" s="2" t="s">
         <v>175</v>
@@ -2479,8 +2589,10 @@
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A57" s="3" t="s">
-        <v>177</v>
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">man</t>
+        </is>
       </c>
       <c r="B57" s="2" t="s">
         <v>178</v>
@@ -2493,8 +2605,10 @@
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A58" s="3" t="s">
-        <v>180</v>
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mother</t>
+        </is>
       </c>
       <c r="B58" s="2" t="s">
         <v>181</v>
@@ -2510,8 +2624,10 @@
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A59" s="3" t="s">
-        <v>183</v>
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mouth</t>
+        </is>
       </c>
       <c r="B59" s="2" t="s">
         <v>184</v>
@@ -2524,8 +2640,10 @@
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A60" s="3" t="s">
-        <v>186</v>
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">much</t>
+        </is>
       </c>
       <c r="B60" s="2" t="s">
         <v>187</v>
@@ -2541,8 +2659,10 @@
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A61" s="3" t="s">
-        <v>189</v>
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">my-child</t>
+        </is>
       </c>
       <c r="B61" s="2" t="s">
         <v>190</v>
@@ -2555,8 +2675,10 @@
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A62" s="3" t="s">
-        <v>193</v>
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">new</t>
+        </is>
       </c>
       <c r="B62" s="2" t="s">
         <v>194</v>
@@ -2572,8 +2694,10 @@
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A63" s="3" t="s">
-        <v>196</v>
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one</t>
+        </is>
       </c>
       <c r="B63" s="2" t="s">
         <v>197</v>
@@ -2586,8 +2710,10 @@
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A64" s="3" t="s">
-        <v>199</v>
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">outside</t>
+        </is>
       </c>
       <c r="B64" s="2" t="s">
         <v>200</v>
@@ -2600,8 +2726,10 @@
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A65" s="3" t="s">
-        <v>202</v>
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">play</t>
+        </is>
       </c>
       <c r="B65" s="2" t="s">
         <v>203</v>
@@ -2614,8 +2742,10 @@
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A66" s="3" t="s">
-        <v>205</v>
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">potato</t>
+        </is>
       </c>
       <c r="B66" s="2" t="s">
         <v>206</v>
@@ -2628,8 +2758,10 @@
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A67" s="3" t="s">
-        <v>208</v>
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">raccoon</t>
+        </is>
       </c>
       <c r="B67" s="2" t="s">
         <v>209</v>
@@ -2642,8 +2774,10 @@
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A68" s="3" t="s">
-        <v>211</v>
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rat</t>
+        </is>
       </c>
       <c r="B68" s="2" t="s">
         <v>212</v>
@@ -2656,8 +2790,10 @@
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A69" s="3" t="s">
-        <v>214</v>
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">road-door</t>
+        </is>
       </c>
       <c r="B69" s="2" t="s">
         <v>215</v>
@@ -2673,8 +2809,10 @@
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A70" s="3" t="s">
-        <v>218</v>
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sack</t>
+        </is>
       </c>
       <c r="B70" s="2" t="s">
         <v>219</v>
@@ -2684,8 +2822,10 @@
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A71" s="3" t="s">
-        <v>220</v>
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scratch</t>
+        </is>
       </c>
       <c r="B71" s="2" t="s">
         <v>221</v>
@@ -2698,8 +2838,10 @@
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A72" s="3" t="s">
-        <v>223</v>
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sheep</t>
+        </is>
       </c>
       <c r="B72" s="2" t="s">
         <v>224</v>
@@ -2712,8 +2854,10 @@
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A73" s="3" t="s">
-        <v>226</v>
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sit-down</t>
+        </is>
       </c>
       <c r="B73" s="2" t="s">
         <v>227</v>
@@ -2726,8 +2870,10 @@
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A74" s="3" t="s">
-        <v>230</v>
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">six</t>
+        </is>
       </c>
       <c r="B74" s="2" t="s">
         <v>231</v>
@@ -2740,8 +2886,10 @@
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A75" s="3" t="s">
-        <v>233</v>
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">skin-hide</t>
+        </is>
       </c>
       <c r="B75" s="2" t="s">
         <v>234</v>
@@ -2754,8 +2902,10 @@
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A76" s="3" t="s">
-        <v>237</v>
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sleep</t>
+        </is>
       </c>
       <c r="B76" s="2" t="s">
         <v>238</v>
@@ -2771,8 +2921,10 @@
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A77" s="3" t="s">
-        <v>240</v>
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">small</t>
+        </is>
       </c>
       <c r="B77" s="2" t="s">
         <v>241</v>
@@ -2788,8 +2940,10 @@
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A78" s="3" t="s">
-        <v>243</v>
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sneezing</t>
+        </is>
       </c>
       <c r="B78" s="2" t="s">
         <v>244</v>
@@ -2802,8 +2956,10 @@
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A79" s="3" t="s">
-        <v>246</v>
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stick</t>
+        </is>
       </c>
       <c r="B79" s="2" t="s">
         <v>247</v>
@@ -2819,8 +2975,10 @@
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A80" s="3" t="s">
-        <v>249</v>
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">strong</t>
+        </is>
       </c>
       <c r="B80" s="2" t="s">
         <v>250</v>
@@ -2836,8 +2994,10 @@
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A81" s="3" t="s">
-        <v>252</v>
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">talking</t>
+        </is>
       </c>
       <c r="B81" s="2" t="s">
         <v>253</v>
@@ -2850,8 +3010,10 @@
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A82" s="3" t="s">
-        <v>255</v>
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ten</t>
+        </is>
       </c>
       <c r="B82" s="2" t="s">
         <v>256</v>
@@ -2864,8 +3026,10 @@
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A83" s="3" t="s">
-        <v>258</v>
+      <c r="A83" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">three</t>
+        </is>
       </c>
       <c r="B83" s="2" t="s">
         <v>259</v>
@@ -2878,8 +3042,10 @@
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A84" s="3" t="s">
-        <v>261</v>
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tide</t>
+        </is>
       </c>
       <c r="B84" s="2" t="s">
         <v>262</v>
@@ -2892,8 +3058,10 @@
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A85" s="3" t="s">
-        <v>264</v>
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tongue</t>
+        </is>
       </c>
       <c r="B85" s="2" t="s">
         <v>265</v>
@@ -2906,8 +3074,10 @@
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A86" s="3" t="s">
-        <v>267</v>
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tooth</t>
+        </is>
       </c>
       <c r="B86" s="2" t="s">
         <v>268</v>
@@ -2920,8 +3090,10 @@
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A87" s="3" t="s">
-        <v>270</v>
+      <c r="A87" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">trying-it</t>
+        </is>
       </c>
       <c r="B87" s="2" t="s">
         <v>321</v>
@@ -2931,8 +3103,10 @@
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A88" s="3" t="s">
-        <v>272</v>
+      <c r="A88" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">uncle-aunt</t>
+        </is>
       </c>
       <c r="B88" s="2" t="s">
         <v>273</v>
@@ -2948,8 +3122,10 @@
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A89" s="3" t="s">
-        <v>276</v>
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">walk</t>
+        </is>
       </c>
       <c r="B89" s="2" t="s">
         <v>277</v>
@@ -2965,8 +3141,10 @@
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A90" s="3" t="s">
-        <v>279</v>
+      <c r="A90" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">water</t>
+        </is>
       </c>
       <c r="B90" s="2" t="s">
         <v>280</v>
@@ -2982,8 +3160,10 @@
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A91" s="3" t="s">
-        <v>282</v>
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">what</t>
+        </is>
       </c>
       <c r="B91" s="2" t="s">
         <v>283</v>
@@ -2996,8 +3176,10 @@
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A92" s="3" t="s">
-        <v>286</v>
+      <c r="A92" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">whistle</t>
+        </is>
       </c>
       <c r="B92" s="2" t="s">
         <v>287</v>
@@ -3010,8 +3192,10 @@
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A93" s="3" t="s">
-        <v>289</v>
+      <c r="A93" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">white</t>
+        </is>
       </c>
       <c r="B93" s="2" t="s">
         <v>290</v>
@@ -3027,8 +3211,10 @@
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A94" s="3" t="s">
-        <v>292</v>
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">white-person</t>
+        </is>
       </c>
       <c r="B94" s="2" t="s">
         <v>293</v>
@@ -3041,8 +3227,10 @@
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A95" s="3" t="s">
-        <v>296</v>
+      <c r="A95" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">who</t>
+        </is>
       </c>
       <c r="B95" s="2" t="s">
         <v>297</v>
@@ -3055,8 +3243,10 @@
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A96" s="3" t="s">
-        <v>300</v>
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">wishing</t>
+        </is>
       </c>
       <c r="B96" s="2" t="s">
         <v>301</v>
@@ -3069,8 +3259,10 @@
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A97" s="3" t="s">
-        <v>303</v>
+      <c r="A97" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
       </c>
       <c r="B97" s="2" t="s">
         <v>304</v>
@@ -3080,8 +3272,10 @@
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A98" s="3" t="s">
-        <v>305</v>
+      <c r="A98" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">you</t>
+        </is>
       </c>
       <c r="B98" s="2" t="s">
         <v>306</v>
@@ -3094,8 +3288,10 @@
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A99" s="3" t="s">
-        <v>308</v>
+      <c r="A99" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">young-woman</t>
+        </is>
       </c>
       <c r="B99" s="2" t="s">
         <v>309</v>
@@ -3111,8 +3307,10 @@
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A100" s="3" t="s">
-        <v>312</v>
+      <c r="A100" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">young-woman-2</t>
+        </is>
       </c>
       <c r="B100" s="2" t="s">
         <v>313</v>
@@ -3125,8 +3323,10 @@
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A101" s="3" t="s">
-        <v>314</v>
+      <c r="A101" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">your-mother</t>
+        </is>
       </c>
       <c r="B101" s="2" t="s">
         <v>315</v>
@@ -3139,8 +3339,10 @@
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A102" s="4" t="s">
-        <v>319</v>
+      <c r="A102" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">two</t>
+        </is>
       </c>
       <c r="B102" s="2" t="s">
         <v>318</v>
@@ -3153,7 +3355,7 @@
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A103" t="inlineStr">
+      <c r="A103" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">run</t>
         </is>
@@ -3169,7 +3371,7 @@
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A104" t="inlineStr">
+      <c r="A104" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">dive</t>
         </is>
@@ -3185,7 +3387,7 @@
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A105" t="inlineStr">
+      <c r="A105" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">fly</t>
         </is>
@@ -3201,7 +3403,7 @@
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A106" t="inlineStr">
+      <c r="A106" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">run-away</t>
         </is>
@@ -3217,7 +3419,7 @@
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A107" t="inlineStr">
+      <c r="A107" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">jump</t>
         </is>
@@ -3233,7 +3435,7 @@
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A108" t="inlineStr">
+      <c r="A108" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">grow</t>
         </is>
@@ -3249,7 +3451,7 @@
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A109" t="inlineStr">
+      <c r="A109" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">get-dressed</t>
         </is>
@@ -3265,7 +3467,7 @@
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A110" t="inlineStr">
+      <c r="A110" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">help-it-him-her-them</t>
         </is>
@@ -3281,7 +3483,7 @@
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A111" t="inlineStr">
+      <c r="A111" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">look-at-it</t>
         </is>
@@ -3297,7 +3499,7 @@
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A112" t="inlineStr">
+      <c r="A112" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">wake-it</t>
         </is>
@@ -3313,7 +3515,7 @@
       </c>
     </row>
     <row r="113" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="A113" t="inlineStr">
+      <c r="A113" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">dry-it</t>
         </is>
@@ -3329,7 +3531,7 @@
       </c>
     </row>
     <row r="114" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="A114" t="inlineStr">
+      <c r="A114" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">hold-it</t>
         </is>
@@ -3345,7 +3547,7 @@
       </c>
     </row>
     <row r="115" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="A115" t="inlineStr">
+      <c r="A115" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">hit-it</t>
         </is>
@@ -3361,7 +3563,7 @@
       </c>
     </row>
     <row r="116" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="A116" t="inlineStr">
+      <c r="A116" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">lift-it</t>
         </is>
@@ -3377,7 +3579,7 @@
       </c>
     </row>
     <row r="117" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="A117" t="inlineStr">
+      <c r="A117" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">choose-it</t>
         </is>
@@ -3393,7 +3595,7 @@
       </c>
     </row>
     <row r="118" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="A118" t="inlineStr">
+      <c r="A118" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">break-it-long-object</t>
         </is>
@@ -3409,7 +3611,7 @@
       </c>
     </row>
     <row r="119" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="A119" t="inlineStr">
+      <c r="A119" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">take-it</t>
         </is>
@@ -3425,7 +3627,7 @@
       </c>
     </row>
     <row r="120" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="A120" t="inlineStr">
+      <c r="A120" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">father</t>
         </is>
@@ -3441,7 +3643,7 @@
       </c>
     </row>
     <row r="121" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="A121" t="inlineStr">
+      <c r="A121" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">money</t>
         </is>
@@ -3457,7 +3659,7 @@
       </c>
     </row>
     <row r="122" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="A122" t="inlineStr">
+      <c r="A122" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">young-man</t>
         </is>
@@ -3473,7 +3675,7 @@
       </c>
     </row>
     <row r="123" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="A123" t="inlineStr">
+      <c r="A123" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">friend</t>
         </is>
@@ -3489,7 +3691,7 @@
       </c>
     </row>
     <row r="124" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="A124" t="inlineStr">
+      <c r="A124" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">word</t>
         </is>
@@ -3505,7 +3707,7 @@
       </c>
     </row>
     <row r="125" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="A125" t="inlineStr">
+      <c r="A125" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">bad</t>
         </is>
@@ -3521,7 +3723,7 @@
       </c>
     </row>
     <row r="126" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="A126" t="inlineStr">
+      <c r="A126" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">old-animate</t>
         </is>
@@ -3537,7 +3739,7 @@
       </c>
     </row>
     <row r="127" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="A127" t="inlineStr">
+      <c r="A127" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">old-worn-out-thing</t>
         </is>
@@ -3553,7 +3755,7 @@
       </c>
     </row>
     <row r="128" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="A128" t="inlineStr">
+      <c r="A128" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">fast</t>
         </is>
@@ -3569,7 +3771,7 @@
       </c>
     </row>
     <row r="129" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="A129" t="inlineStr">
+      <c r="A129" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">i-intransitive</t>
         </is>
@@ -3585,7 +3787,7 @@
       </c>
     </row>
     <row r="130" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="A130" t="inlineStr">
+      <c r="A130" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">we-intransitive</t>
         </is>
@@ -3601,7 +3803,7 @@
       </c>
     </row>
     <row r="131" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="A131" t="inlineStr">
+      <c r="A131" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">you-intransitive</t>
         </is>
@@ -3617,7 +3819,7 @@
       </c>
     </row>
     <row r="132" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="A132" t="inlineStr">
+      <c r="A132" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">you-all-you-folks-intransitive</t>
         </is>
@@ -3633,7 +3835,7 @@
       </c>
     </row>
     <row r="133" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="A133" t="inlineStr">
+      <c r="A133" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">he-she-it-they-transitive-suffix</t>
         </is>
@@ -3649,7 +3851,7 @@
       </c>
     </row>
     <row r="134" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="A134" t="inlineStr">
+      <c r="A134" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">the-that-specific-article</t>
         </is>
@@ -3665,7 +3867,7 @@
       </c>
     </row>
     <row r="135" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="A135" t="inlineStr">
+      <c r="A135" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">your</t>
         </is>
@@ -3678,7 +3880,7 @@
       </c>
     </row>
     <row r="136" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="A136" t="inlineStr">
+      <c r="A136" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">work</t>
         </is>
@@ -3691,7 +3893,7 @@
       </c>
     </row>
     <row r="137" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="A137" t="inlineStr">
+      <c r="A137" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">salt</t>
         </is>
@@ -3704,7 +3906,7 @@
       </c>
     </row>
     <row r="138" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="A138" t="inlineStr">
+      <c r="A138" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">raven</t>
         </is>
@@ -3717,7 +3919,7 @@
       </c>
     </row>
     <row r="139" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="A139" t="inlineStr">
+      <c r="A139" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">grandparent</t>
         </is>

</xml_diff>